<commit_message>
Added mappers for medicine dto. added ExcelExporter, ExcelTemplateFiller
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/excel/medicine.xlsx
+++ b/src/main/resources/templates/excel/medicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\java\XRC_new\exporter\rad-exporter\src\main\resources\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62A9E1E4-0791-447B-A05A-F8E73A9D99FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26E9399-EF16-4CCC-92D6-E9517AF97268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="4800" windowWidth="29040" windowHeight="16440" xr2:uid="{7DF7E526-0462-4853-B29A-D1AED53DCF3C}"/>
   </bookViews>
@@ -20,8 +20,8 @@
     <definedName name="deviceProtection">Лист1!$A$19:$B$19</definedName>
     <definedName name="material">Лист1!$A$16:$B$18</definedName>
     <definedName name="openings">Лист1!$A$23</definedName>
-    <definedName name="panel">Лист1!$C$7:$C$26</definedName>
-    <definedName name="protectionTable">Лист1!$A$2:$C$26</definedName>
+    <definedName name="panel">Лист1!$C$7:$C$24</definedName>
+    <definedName name="protectionTable">Лист1!$A$2:$C$24</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>Расчёт защиты от рентгеновского излучения для аппарата: $device.name</t>
   </si>
@@ -322,15 +322,6 @@
     <t>$pbEquivalent$</t>
   </si>
   <si>
-    <t>$exMatName$</t>
-  </si>
-  <si>
-    <t>$exMatThick$</t>
-  </si>
-  <si>
-    <t>$exMatLead$</t>
-  </si>
-  <si>
     <t>$deviceLead$</t>
   </si>
   <si>
@@ -343,19 +334,22 @@
     <t>$demandMatThickness$</t>
   </si>
   <si>
-    <t>$opening1Name$</t>
-  </si>
-  <si>
-    <t>$opening1Lead$</t>
-  </si>
-  <si>
-    <t>$opening2Lead$</t>
-  </si>
-  <si>
-    <t>$opening2Name$</t>
-  </si>
-  <si>
     <t>$roomPurpose$</t>
+  </si>
+  <si>
+    <t>$exMatName0$</t>
+  </si>
+  <si>
+    <t>$exMatThick0$</t>
+  </si>
+  <si>
+    <t>$exMatLead0$</t>
+  </si>
+  <si>
+    <t>$openingName0$</t>
+  </si>
+  <si>
+    <t>$openingLead0$</t>
   </si>
 </sst>
 </file>
@@ -624,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -655,6 +649,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -671,24 +680,6 @@
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1004,7 +995,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B1CCD8-9D2C-4D57-99AE-C6AEBCFD7404}">
-  <dimension ref="A2:C27"/>
+  <dimension ref="A2:C24"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="26.3515625" style="1" customWidth="1"/>
@@ -1035,113 +1026,113 @@
     </row>
     <row r="6" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6"/>
     <row r="7" spans="1:3" ht="16.350000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="12"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="14"/>
+      <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="14"/>
+      <c r="B9" s="19"/>
       <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="19"/>
       <c r="C10" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="19"/>
       <c r="C11" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30.7" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="12"/>
+      <c r="B13" s="17"/>
       <c r="C13" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="14"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="70" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A17" s="18"/>
+      <c r="A17" s="13"/>
       <c r="B17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="19"/>
+      <c r="A18" s="15"/>
       <c r="B18" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="50" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
@@ -1152,72 +1143,57 @@
         <v>16</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="50" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="80" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A21" s="18"/>
+      <c r="A21" s="13"/>
       <c r="B21" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="19"/>
+      <c r="A22" s="15"/>
       <c r="B22" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="16.350000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="20"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A24" s="18"/>
-      <c r="B24" s="21"/>
+      <c r="A24" s="13"/>
+      <c r="B24" s="14"/>
       <c r="C24" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A25" s="18"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A26" s="19"/>
-      <c r="B26" s="22"/>
-      <c r="C26" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="16" thickTop="1" x14ac:dyDescent="0.55000000000000004"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A23:B26"/>
+    <mergeCell ref="A23:B24"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>

</xml_diff>